<commit_message>
update data prep and controls pages
</commit_message>
<xml_diff>
--- a/raw data/aux_data.xlsx
+++ b/raw data/aux_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Microbiome_Analysis_Workflow\raw data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843025E6-F733-4783-AD56-97B5BACC2A3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{091E8852-1F6B-4806-9FEA-A513D835C415}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="2520" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -38,6 +38,40 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Karelle Rheault</author>
+  </authors>
+  <commentList>
+    <comment ref="A74" authorId="0" shapeId="0" xr:uid="{F28D2A7F-1A6E-4E5A-BEC4-C075BD7F9535}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Karelle Rheault:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Low LibrarySize sample</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Karelle Rheault</author>
@@ -97,7 +131,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="554">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="552">
   <si>
     <t>Site</t>
   </si>
@@ -1830,16 +1864,10 @@
     <t>SNF5__29245</t>
   </si>
   <si>
-    <t>Spruce</t>
-  </si>
-  <si>
     <t>732a</t>
   </si>
   <si>
-    <t>Spruce_52</t>
-  </si>
-  <si>
-    <t>Spruce_52_B</t>
+    <t>Oak_51_B</t>
   </si>
 </sst>
 </file>
@@ -1850,7 +1878,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1901,6 +1929,19 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -2286,41 +2327,41 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AC101"/>
-  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="7.81640625" customWidth="1"/>
-    <col min="2" max="2" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.36328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.54296875" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.77734375" customWidth="1"/>
+    <col min="2" max="2" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.77734375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.77734375" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="6.81640625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="5.08984375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="6.36328125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="6.54296875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="6.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:29" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2409,7 +2450,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>46</v>
       </c>
@@ -2495,7 +2536,7 @@
         <v>0.25669100746770301</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -2581,7 +2622,7 @@
         <v>0.25669100746770301</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -2667,7 +2708,7 @@
         <v>0.25669100746770301</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -2753,7 +2794,7 @@
         <v>0.25669100746770301</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>46</v>
       </c>
@@ -2839,7 +2880,7 @@
         <v>0.25669100746770301</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -2925,7 +2966,7 @@
         <v>0.25669100746770301</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -3011,7 +3052,7 @@
         <v>0.25669100746770301</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>46</v>
       </c>
@@ -3097,7 +3138,7 @@
         <v>0.25669100746770301</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>46</v>
       </c>
@@ -3183,7 +3224,7 @@
         <v>0.25669100746770301</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -3269,7 +3310,7 @@
         <v>0.156012375633622</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -3355,7 +3396,7 @@
         <v>0.156012375633622</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -3441,7 +3482,7 @@
         <v>0.156012375633622</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>25</v>
       </c>
@@ -3527,7 +3568,7 @@
         <v>0.156012375633622</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -3613,7 +3654,7 @@
         <v>0.156012375633622</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -3699,7 +3740,7 @@
         <v>0.156012375633622</v>
       </c>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>25</v>
       </c>
@@ -3785,7 +3826,7 @@
         <v>0.156012375633622</v>
       </c>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>25</v>
       </c>
@@ -3871,7 +3912,7 @@
         <v>0.156012375633622</v>
       </c>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>25</v>
       </c>
@@ -3957,7 +3998,7 @@
         <v>0.156012375633622</v>
       </c>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>40</v>
       </c>
@@ -4046,7 +4087,7 @@
         <v>0.455637451007188</v>
       </c>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>40</v>
       </c>
@@ -4135,7 +4176,7 @@
         <v>0.455637451007188</v>
       </c>
     </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -4224,7 +4265,7 @@
         <v>0.455637451007188</v>
       </c>
     </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -4313,7 +4354,7 @@
         <v>0.455637451007188</v>
       </c>
     </row>
-    <row r="24" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>40</v>
       </c>
@@ -4402,7 +4443,7 @@
         <v>0.455637451007188</v>
       </c>
     </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>40</v>
       </c>
@@ -4491,7 +4532,7 @@
         <v>0.455637451007188</v>
       </c>
     </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>40</v>
       </c>
@@ -4580,7 +4621,7 @@
         <v>0.455637451007188</v>
       </c>
     </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -4669,7 +4710,7 @@
         <v>0.455637451007188</v>
       </c>
     </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -4758,7 +4799,7 @@
         <v>0.455637451007188</v>
       </c>
     </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>42</v>
       </c>
@@ -4847,7 +4888,7 @@
         <v>0.49056697904695301</v>
       </c>
     </row>
-    <row r="30" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -4936,7 +4977,7 @@
         <v>0.49056697904695301</v>
       </c>
     </row>
-    <row r="31" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>42</v>
       </c>
@@ -5025,7 +5066,7 @@
         <v>0.49056697904695301</v>
       </c>
     </row>
-    <row r="32" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -5114,7 +5155,7 @@
         <v>0.49056697904695301</v>
       </c>
     </row>
-    <row r="33" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>42</v>
       </c>
@@ -5203,7 +5244,7 @@
         <v>0.49056697904695301</v>
       </c>
     </row>
-    <row r="34" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>42</v>
       </c>
@@ -5292,7 +5333,7 @@
         <v>0.49056697904695301</v>
       </c>
     </row>
-    <row r="35" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>42</v>
       </c>
@@ -5381,7 +5422,7 @@
         <v>0.49056697904695301</v>
       </c>
     </row>
-    <row r="36" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -5470,7 +5511,7 @@
         <v>0.49056697904695301</v>
       </c>
     </row>
-    <row r="37" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -5559,7 +5600,7 @@
         <v>0.49056697904695301</v>
       </c>
     </row>
-    <row r="38" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -5648,7 +5689,7 @@
         <v>0.42960470863432898</v>
       </c>
     </row>
-    <row r="39" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>39</v>
       </c>
@@ -5737,7 +5778,7 @@
         <v>0.42960470863432898</v>
       </c>
     </row>
-    <row r="40" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -5826,7 +5867,7 @@
         <v>0.42960470863432898</v>
       </c>
     </row>
-    <row r="41" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -5915,7 +5956,7 @@
         <v>0.42960470863432898</v>
       </c>
     </row>
-    <row r="42" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>39</v>
       </c>
@@ -6004,7 +6045,7 @@
         <v>0.42960470863432898</v>
       </c>
     </row>
-    <row r="43" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>39</v>
       </c>
@@ -6093,7 +6134,7 @@
         <v>0.42960470863432898</v>
       </c>
     </row>
-    <row r="44" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>39</v>
       </c>
@@ -6182,7 +6223,7 @@
         <v>0.42960470863432898</v>
       </c>
     </row>
-    <row r="45" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>39</v>
       </c>
@@ -6271,7 +6312,7 @@
         <v>0.42960470863432898</v>
       </c>
     </row>
-    <row r="46" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>39</v>
       </c>
@@ -6360,7 +6401,7 @@
         <v>0.42960470863432898</v>
       </c>
     </row>
-    <row r="47" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>45</v>
       </c>
@@ -6449,7 +6490,7 @@
         <v>0.29560986108328802</v>
       </c>
     </row>
-    <row r="48" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>45</v>
       </c>
@@ -6538,7 +6579,7 @@
         <v>0.29560986108328802</v>
       </c>
     </row>
-    <row r="49" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>45</v>
       </c>
@@ -6627,7 +6668,7 @@
         <v>0.29560986108328802</v>
       </c>
     </row>
-    <row r="50" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>45</v>
       </c>
@@ -6716,7 +6757,7 @@
         <v>0.29560986108328802</v>
       </c>
     </row>
-    <row r="51" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>45</v>
       </c>
@@ -6805,7 +6846,7 @@
         <v>0.29560986108328802</v>
       </c>
     </row>
-    <row r="52" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>45</v>
       </c>
@@ -6894,7 +6935,7 @@
         <v>0.29560986108328802</v>
       </c>
     </row>
-    <row r="53" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>45</v>
       </c>
@@ -6983,7 +7024,7 @@
         <v>0.29560986108328802</v>
       </c>
     </row>
-    <row r="54" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>45</v>
       </c>
@@ -7072,7 +7113,7 @@
         <v>0.29560986108328802</v>
       </c>
     </row>
-    <row r="55" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>45</v>
       </c>
@@ -7161,7 +7202,7 @@
         <v>0.29560986108328802</v>
       </c>
     </row>
-    <row r="56" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>43</v>
       </c>
@@ -7250,7 +7291,7 @@
         <v>0.30029290148423399</v>
       </c>
     </row>
-    <row r="57" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>43</v>
       </c>
@@ -7339,7 +7380,7 @@
         <v>0.30029290148423399</v>
       </c>
     </row>
-    <row r="58" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>43</v>
       </c>
@@ -7428,7 +7469,7 @@
         <v>0.30029290148423399</v>
       </c>
     </row>
-    <row r="59" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>43</v>
       </c>
@@ -7517,7 +7558,7 @@
         <v>0.30029290148423399</v>
       </c>
     </row>
-    <row r="60" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>43</v>
       </c>
@@ -7606,7 +7647,7 @@
         <v>0.30029290148423399</v>
       </c>
     </row>
-    <row r="61" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>43</v>
       </c>
@@ -7695,7 +7736,7 @@
         <v>0.30029290148423399</v>
       </c>
     </row>
-    <row r="62" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>43</v>
       </c>
@@ -7784,7 +7825,7 @@
         <v>0.30029290148423399</v>
       </c>
     </row>
-    <row r="63" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>43</v>
       </c>
@@ -7873,7 +7914,7 @@
         <v>0.30029290148423399</v>
       </c>
     </row>
-    <row r="64" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>43</v>
       </c>
@@ -7962,7 +8003,7 @@
         <v>0.30029290148423399</v>
       </c>
     </row>
-    <row r="65" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>41</v>
       </c>
@@ -8051,7 +8092,7 @@
         <v>0.26149340192385301</v>
       </c>
     </row>
-    <row r="66" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>41</v>
       </c>
@@ -8140,7 +8181,7 @@
         <v>0.26149340192385301</v>
       </c>
     </row>
-    <row r="67" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>41</v>
       </c>
@@ -8229,7 +8270,7 @@
         <v>0.26149340192385301</v>
       </c>
     </row>
-    <row r="68" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>41</v>
       </c>
@@ -8318,7 +8359,7 @@
         <v>0.26149340192385301</v>
       </c>
     </row>
-    <row r="69" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>41</v>
       </c>
@@ -8407,7 +8448,7 @@
         <v>0.26149340192385301</v>
       </c>
     </row>
-    <row r="70" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>41</v>
       </c>
@@ -8496,7 +8537,7 @@
         <v>0.26149340192385301</v>
       </c>
     </row>
-    <row r="71" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>41</v>
       </c>
@@ -8585,7 +8626,7 @@
         <v>0.26149340192385301</v>
       </c>
     </row>
-    <row r="72" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>41</v>
       </c>
@@ -8674,7 +8715,7 @@
         <v>0.26149340192385301</v>
       </c>
     </row>
-    <row r="73" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>41</v>
       </c>
@@ -8763,30 +8804,30 @@
         <v>0.26149340192385301</v>
       </c>
     </row>
-    <row r="74" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B74" t="s">
         <v>10</v>
       </c>
       <c r="C74" t="s">
-        <v>552</v>
+        <v>58</v>
       </c>
       <c r="D74" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="E74" t="s">
-        <v>550</v>
+        <v>38</v>
       </c>
       <c r="F74" t="s">
-        <v>550</v>
+        <v>38</v>
       </c>
       <c r="G74">
-        <v>1969</v>
+        <v>1970</v>
       </c>
       <c r="H74">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I74" t="s">
         <v>425</v>
@@ -8853,7 +8894,7 @@
         <v>0.58050172170519221</v>
       </c>
     </row>
-    <row r="75" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>37</v>
       </c>
@@ -8942,7 +8983,7 @@
         <v>0.201206586059272</v>
       </c>
     </row>
-    <row r="76" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>37</v>
       </c>
@@ -9031,7 +9072,7 @@
         <v>0.201206586059272</v>
       </c>
     </row>
-    <row r="77" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>37</v>
       </c>
@@ -9120,7 +9161,7 @@
         <v>0.201206586059272</v>
       </c>
     </row>
-    <row r="78" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>37</v>
       </c>
@@ -9209,7 +9250,7 @@
         <v>0.201206586059272</v>
       </c>
     </row>
-    <row r="79" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>37</v>
       </c>
@@ -9298,7 +9339,7 @@
         <v>0.201206586059272</v>
       </c>
     </row>
-    <row r="80" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>37</v>
       </c>
@@ -9387,7 +9428,7 @@
         <v>0.201206586059272</v>
       </c>
     </row>
-    <row r="81" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>37</v>
       </c>
@@ -9476,7 +9517,7 @@
         <v>0.201206586059272</v>
       </c>
     </row>
-    <row r="82" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>37</v>
       </c>
@@ -9565,7 +9606,7 @@
         <v>0.201206586059272</v>
       </c>
     </row>
-    <row r="83" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>37</v>
       </c>
@@ -9654,7 +9695,7 @@
         <v>0.201206586059272</v>
       </c>
     </row>
-    <row r="84" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>48</v>
       </c>
@@ -9743,7 +9784,7 @@
         <v>0.56153801714094498</v>
       </c>
     </row>
-    <row r="85" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>48</v>
       </c>
@@ -9832,7 +9873,7 @@
         <v>0.56153801714094498</v>
       </c>
     </row>
-    <row r="86" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>48</v>
       </c>
@@ -9921,7 +9962,7 @@
         <v>0.56153801714094498</v>
       </c>
     </row>
-    <row r="87" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>48</v>
       </c>
@@ -10010,7 +10051,7 @@
         <v>0.56153801714094498</v>
       </c>
     </row>
-    <row r="88" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>48</v>
       </c>
@@ -10099,7 +10140,7 @@
         <v>0.56153801714094498</v>
       </c>
     </row>
-    <row r="89" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>48</v>
       </c>
@@ -10188,7 +10229,7 @@
         <v>0.56153801714094498</v>
       </c>
     </row>
-    <row r="90" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>48</v>
       </c>
@@ -10277,7 +10318,7 @@
         <v>0.56153801714094498</v>
       </c>
     </row>
-    <row r="91" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>48</v>
       </c>
@@ -10366,7 +10407,7 @@
         <v>0.56153801714094498</v>
       </c>
     </row>
-    <row r="92" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>48</v>
       </c>
@@ -10455,7 +10496,7 @@
         <v>0.56153801714094498</v>
       </c>
     </row>
-    <row r="93" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:29" x14ac:dyDescent="0.3">
       <c r="I93" t="s">
         <v>273</v>
       </c>
@@ -10466,7 +10507,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="94" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:29" x14ac:dyDescent="0.3">
       <c r="I94" t="s">
         <v>406</v>
       </c>
@@ -10477,7 +10518,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="95" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:29" x14ac:dyDescent="0.3">
       <c r="I95" t="s">
         <v>276</v>
       </c>
@@ -10488,7 +10529,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="96" spans="1:29" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:29" x14ac:dyDescent="0.3">
       <c r="I96" t="s">
         <v>277</v>
       </c>
@@ -10499,7 +10540,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="97" spans="9:11" x14ac:dyDescent="0.35">
+    <row r="97" spans="9:11" x14ac:dyDescent="0.3">
       <c r="I97" t="s">
         <v>278</v>
       </c>
@@ -10510,7 +10551,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="98" spans="9:11" x14ac:dyDescent="0.35">
+    <row r="98" spans="9:11" x14ac:dyDescent="0.3">
       <c r="I98" t="s">
         <v>272</v>
       </c>
@@ -10521,7 +10562,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="99" spans="9:11" x14ac:dyDescent="0.35">
+    <row r="99" spans="9:11" x14ac:dyDescent="0.3">
       <c r="I99" t="s">
         <v>275</v>
       </c>
@@ -10532,7 +10573,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="100" spans="9:11" x14ac:dyDescent="0.35">
+    <row r="100" spans="9:11" x14ac:dyDescent="0.3">
       <c r="I100" t="s">
         <v>274</v>
       </c>
@@ -10543,7 +10584,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="101" spans="9:11" x14ac:dyDescent="0.35">
+    <row r="101" spans="9:11" x14ac:dyDescent="0.3">
       <c r="I101" t="s">
         <v>279</v>
       </c>
@@ -10563,30 +10604,31 @@
   <conditionalFormatting sqref="I1:I100 I102:I1048576">
     <cfRule type="duplicateValues" dxfId="5" priority="4"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I101">
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J1:J100 J102:J1048576">
-    <cfRule type="duplicateValues" dxfId="4" priority="3"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I101">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J101">
     <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D9B7D62-E9F1-4792-8EF4-33F7CA42B523}">
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="11.54296875" customWidth="1"/>
-    <col min="4" max="4" width="14.54296875" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>152</v>
       </c>
@@ -10600,7 +10642,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -10611,7 +10653,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -10622,7 +10664,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -10636,7 +10678,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>23</v>
       </c>
@@ -10650,7 +10692,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -10664,7 +10706,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -10675,7 +10717,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -10686,7 +10728,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -10697,7 +10739,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -10708,7 +10750,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -10719,7 +10761,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -10730,7 +10772,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -10741,7 +10783,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -10752,7 +10794,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -10763,7 +10805,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -10774,7 +10816,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -10782,7 +10824,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>170</v>
       </c>
@@ -10799,14 +10841,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56344B17-448D-448F-96FD-4901AF1E2959}">
   <dimension ref="A1:C87"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
@@ -10817,7 +10859,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>407</v>
       </c>
@@ -10828,7 +10870,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>408</v>
       </c>
@@ -10839,7 +10881,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>409</v>
       </c>
@@ -10850,7 +10892,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>410</v>
       </c>
@@ -10861,7 +10903,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>411</v>
       </c>
@@ -10872,7 +10914,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>412</v>
       </c>
@@ -10883,7 +10925,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>374</v>
       </c>
@@ -10894,7 +10936,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>375</v>
       </c>
@@ -10905,7 +10947,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>376</v>
       </c>
@@ -10916,7 +10958,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>413</v>
       </c>
@@ -10927,7 +10969,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>414</v>
       </c>
@@ -10938,7 +10980,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>415</v>
       </c>
@@ -10949,7 +10991,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>416</v>
       </c>
@@ -10960,7 +11002,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>417</v>
       </c>
@@ -10971,7 +11013,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>389</v>
       </c>
@@ -10982,7 +11024,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>418</v>
       </c>
@@ -10993,7 +11035,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>419</v>
       </c>
@@ -11004,7 +11046,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>420</v>
       </c>
@@ -11015,7 +11057,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>421</v>
       </c>
@@ -11026,7 +11068,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>422</v>
       </c>
@@ -11037,7 +11079,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>423</v>
       </c>
@@ -11048,7 +11090,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>424</v>
       </c>
@@ -11059,7 +11101,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>426</v>
       </c>
@@ -11070,7 +11112,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>427</v>
       </c>
@@ -11081,7 +11123,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>428</v>
       </c>
@@ -11092,7 +11134,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>377</v>
       </c>
@@ -11103,7 +11145,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>429</v>
       </c>
@@ -11114,7 +11156,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>378</v>
       </c>
@@ -11125,7 +11167,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>430</v>
       </c>
@@ -11136,7 +11178,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>379</v>
       </c>
@@ -11147,7 +11189,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>380</v>
       </c>
@@ -11158,7 +11200,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>381</v>
       </c>
@@ -11169,7 +11211,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>382</v>
       </c>
@@ -11180,7 +11222,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>431</v>
       </c>
@@ -11191,7 +11233,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>432</v>
       </c>
@@ -11202,7 +11244,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>383</v>
       </c>
@@ -11213,7 +11255,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>433</v>
       </c>
@@ -11224,7 +11266,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>434</v>
       </c>
@@ -11235,7 +11277,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>384</v>
       </c>
@@ -11246,7 +11288,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>385</v>
       </c>
@@ -11257,7 +11299,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>386</v>
       </c>
@@ -11268,7 +11310,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>404</v>
       </c>
@@ -11279,7 +11321,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>387</v>
       </c>
@@ -11290,7 +11332,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>388</v>
       </c>
@@ -11301,7 +11343,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>405</v>
       </c>
@@ -11312,7 +11354,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>390</v>
       </c>
@@ -11323,7 +11365,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>435</v>
       </c>
@@ -11334,7 +11376,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>391</v>
       </c>
@@ -11345,7 +11387,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>436</v>
       </c>
@@ -11356,7 +11398,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>392</v>
       </c>
@@ -11367,7 +11409,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>437</v>
       </c>
@@ -11378,7 +11420,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>393</v>
       </c>
@@ -11389,7 +11431,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>438</v>
       </c>
@@ -11400,7 +11442,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>439</v>
       </c>
@@ -11411,7 +11453,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>440</v>
       </c>
@@ -11422,7 +11464,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>441</v>
       </c>
@@ -11433,7 +11475,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>394</v>
       </c>
@@ -11444,7 +11486,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>395</v>
       </c>
@@ -11455,7 +11497,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>442</v>
       </c>
@@ -11466,7 +11508,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>396</v>
       </c>
@@ -11477,7 +11519,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>443</v>
       </c>
@@ -11488,7 +11530,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>444</v>
       </c>
@@ -11499,7 +11541,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>445</v>
       </c>
@@ -11510,7 +11552,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>446</v>
       </c>
@@ -11521,7 +11563,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>397</v>
       </c>
@@ -11532,7 +11574,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>447</v>
       </c>
@@ -11543,7 +11585,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>448</v>
       </c>
@@ -11554,7 +11596,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>449</v>
       </c>
@@ -11565,7 +11607,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>450</v>
       </c>
@@ -11576,7 +11618,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>451</v>
       </c>
@@ -11587,7 +11629,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>452</v>
       </c>
@@ -11598,7 +11640,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>398</v>
       </c>
@@ -11609,7 +11651,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>399</v>
       </c>
@@ -11620,7 +11662,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>453</v>
       </c>
@@ -11631,7 +11673,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>454</v>
       </c>
@@ -11642,7 +11684,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>455</v>
       </c>
@@ -11653,7 +11695,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>400</v>
       </c>
@@ -11664,7 +11706,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>456</v>
       </c>
@@ -11675,7 +11717,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>457</v>
       </c>
@@ -11686,7 +11728,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>401</v>
       </c>
@@ -11697,7 +11739,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>402</v>
       </c>
@@ -11708,7 +11750,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>458</v>
       </c>
@@ -11719,7 +11761,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>459</v>
       </c>
@@ -11730,7 +11772,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>403</v>
       </c>
@@ -11741,7 +11783,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>460</v>
       </c>
@@ -11752,7 +11794,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>461</v>
       </c>

</xml_diff>